<commit_message>
Verified: Tindak Lanjut, Simpan Dashboard, History semua berfungsi
- Tindak Lanjut: 6 aspek dari sheet Excel (Eskalasi, Tim & Peran,
  Pesan & Kanal, Eksekusi, Evaluasi, Esensi) x 3 Tier, highlight
  kolom tier aktif berdasarkan rata-rata IIRS
- Simpan Dashboard (admin only): menyimpan snapshot ke history.json
  dengan timestamp ISO untuk retensi 7 hari
- History (admin only): list snapshot, view, hapus, badge expires
- Uploader: tidak bisa akses simpan/history

https://claude.ai/code/session_012KajSB15QHs2faZ4YuFhrV
</commit_message>
<xml_diff>
--- a/iirs_app/uploads/latest.xlsx
+++ b/iirs_app/uploads/latest.xlsx
@@ -5,18 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bankindonesiagov-my.sharepoint.com/personal/hilmy_munis_bi_go_id/Documents/SESMUBI 2026/Final Project Kelompok 14/Analisis DATA BAB 4 IIRS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Rino\LEARNING\SESMU_15_2026\FINAL_PROJECT\TUGAS\130526\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="125" documentId="13_ncr:1_{13A1985F-C9FA-47ED-B1BC-7375BFE6E13A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A2F510A-2109-4613-B784-F85864BBB2A0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3808BA66-E405-4F99-A000-D2310CF6DE10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D9861903-4DD6-443F-BDCB-8CE2F4A777AE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="4" xr2:uid="{D9861903-4DD6-443F-BDCB-8CE2F4A777AE}"/>
   </bookViews>
   <sheets>
     <sheet name="GET THINGS DONE!" sheetId="4" r:id="rId1"/>
     <sheet name="Source Scoring" sheetId="1" r:id="rId2"/>
     <sheet name="IIRS Integration" sheetId="2" r:id="rId3"/>
     <sheet name="Indikator EWS" sheetId="3" r:id="rId4"/>
+    <sheet name="Tindak Lanjut" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'IIRS Integration'!$A$3:$G$6</definedName>
@@ -81,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="89">
   <si>
     <t>Source Score Data</t>
   </si>
@@ -167,15 +168,6 @@
   </si>
   <si>
     <t>Indikator EWS</t>
-  </si>
-  <si>
-    <t>Playbook 1</t>
-  </si>
-  <si>
-    <t>Playbook 2</t>
-  </si>
-  <si>
-    <t>Playbook 3</t>
   </si>
   <si>
     <t>Pengerjaan periode 13 (Rabu) s.d. 16 (Sabtu) 2026</t>
@@ -256,12 +248,123 @@
   <si>
     <t>https://claude.ai/share/311a631d-7edd-431a-bfd1-b97a5664f052</t>
   </si>
+  <si>
+    <t xml:space="preserve"> Panduan Respons 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Panduan Respons 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Panduan Respons 3</t>
+  </si>
+  <si>
+    <t>Aspek</t>
+  </si>
+  <si>
+    <t>Tier 1 — Ringan (IIRS 0–35)</t>
+  </si>
+  <si>
+    <t>Tier 2 — Sedang (IIRS 36–59)</t>
+  </si>
+  <si>
+    <t>Tier 3 — Crisis (IIRS ≥60)</t>
+  </si>
+  <si>
+    <t>1. Eskalasi</t>
+  </si>
+  <si>
+    <t>DP2K &amp; DLIPKD memantau dua sumber secara paralel (Sentrix + No Limit); laporan mingguan terintegrasi ke Kepala Divisi DKom.</t>
+  </si>
+  <si>
+    <t>SLA: maksimum 24 jam.</t>
+  </si>
+  <si>
+    <t>Joint issue brief DP2K–DLIPKD ke Kepala Grup + Kepala Satker DKom; dibawa ke RDG Mingguan sebagai early heads-up ke forum BI-WIDE.</t>
+  </si>
+  <si>
+    <t>Fase siaga (IIRS 50–59): eskalasi diperluas ke DKEM, DKMP, DKSP, dan satker lain.</t>
+  </si>
+  <si>
+    <t>SLA: maksimum 12 jam.</t>
+  </si>
+  <si>
+    <t>Executive brief DP2K–DLIPKD ke ADG bidang; isu menjadi agenda khusus RDG Mingguan bersama Kepala Satker DKom, Kepala Departemen terkait, ADG, dan Gubernur BI.</t>
+  </si>
+  <si>
+    <t>SLA: maksimum 6 jam.</t>
+  </si>
+  <si>
+    <t>2. Tim &amp; Peran</t>
+  </si>
+  <si>
+    <t>DP2K: pemilik insight utama, menerjemahkan IIRS menjadi tema komunikasi bulanan. DLIPKD: wakil koordinator insight + eksekutor media digital. DROM: relasi rutin wartawan &amp; KOL. TRPI: cascading tema ke 46 KPwDN.</t>
+  </si>
+  <si>
+    <t>DP2K &amp; DLIPKD sebagai joint issue owner (sisi Non-Kanal &amp; Kanal BI). DROM mengintensifkan KOL engagement + taklimat tematik. TRPI mengoordinasikan synchronized posting 46 KPwDN.</t>
+  </si>
+  <si>
+    <t>Juru Bicara: Kepala Grup. Otoritas pemutus: Kepala Satker DKom.</t>
+  </si>
+  <si>
+    <t>DP2K merumuskan arah pesan multi-minggu ke Crisis Management Committee. DLIPKD memproduksi konten penuh di 6 kanal + kemitraan. DROM memfasilitasi press conference &amp; KOL coalition. TRPI mengaktivasi penuh 46 KPwDN sebagai frontline regional.</t>
+  </si>
+  <si>
+    <t>Juru Bicara: ADG/Gubernur BI; layer ke-2: Kepala DKom.</t>
+  </si>
+  <si>
+    <t>3. Pesan &amp; Kanal</t>
+  </si>
+  <si>
+    <t>Pendekatan edukasi proaktif. Konten organik edukatif (evergreen) di kanal BI, ditopang paid promotion ringan. Taklimat media bulanan reguler pasca-RDG. 46 KPwDN memposting tema bulanan seragam dengan kreativitas lokal.</t>
+  </si>
+  <si>
+    <t>Klarifikasi reaktif + edukasi tematik intensif. Key message tiga lapis: penegasan faktual → klarifikasi konteks → edukasi mendalam. Paid promotion diperbesar + aktivasi influencer/kreator &amp; clipper. KOL ekonom sebagai secondary amplifier. 46 KPwDN melakukan echoing narasi inti.</t>
+  </si>
+  <si>
+    <t>Crisis containment penuh + menjaga kredibilitas. Official statement Dewan Gubernur + Q&amp;A lengkap. Seluruh 6 kanal kapasitas penuh + paid promotion maksimal + koalisi kemitraan. Press conference ADG/Gubernur + town hall. 46 KPwDN mendorong advocate GenBI, akademisi, UMKM, dan mitra strategis daerah.</t>
+  </si>
+  <si>
+    <t>4. Eksekusi &amp; Koordinasi</t>
+  </si>
+  <si>
+    <t>Posting konten terjadwal sesuai content plan DLIPKD. Koordinasi internal DKom melalui forum Rapat Redaksi.</t>
+  </si>
+  <si>
+    <t>Rolling content mingguan dengan A/B testing narasi; pemantauan dua sisi (DP2K mengawasi Non-Kanal BI, DLIPKD mengawasi Kanal BI). DP2K sebagai intelligence center. Koordinasi awal dengan satker substansi (DKEM/DKMP/DKSP) untuk validasi konten teknis.</t>
+  </si>
+  <si>
+    <t>Pemantauan harian; laporan kondisi eksternal dan kanal BI disampaikan bersamaan agar Committee dapat langsung membandingkan kedua kondisi. Koordinasi seluruh departemen relevan + KSSK (Kemenkeu/OJK/LPS); briefing DPR Komisi XI bila diperlukan.</t>
+  </si>
+  <si>
+    <t>5. Evaluasi &amp; Pembelajaran</t>
+  </si>
+  <si>
+    <t>Review bulanan oleh Kepala Divisi terkait; laporan IIRS dua perspektif menjadi input tema berikutnya. De-eskalasi: tier dasar — naik ke Tier 2 bila IIRS melewati 35.</t>
+  </si>
+  <si>
+    <t>Weekly review; laporan bersama DP2K–DLIPKD ke RDG Mingguan. De-eskalasi: turun ke Tier 1 bila IIRS stabil di bawah 36, disahkan Kepala Divisi terkait.</t>
+  </si>
+  <si>
+    <t>Daily review; laporan bersama ke ADG bidang/Gubernur BI. De-eskalasi: turun ke Tier 2 bila IIRS stabil di bawah 60, disahkan Kepala Satker DKom. Feedback Loop menjadi input kalibrasi batas tier &amp; crisis simulation drill.</t>
+  </si>
+  <si>
+    <t>Esensi</t>
+  </si>
+  <si>
+    <t>Active baseline maintenance</t>
+  </si>
+  <si>
+    <t>Proactive control</t>
+  </si>
+  <si>
+    <t>Credibility preservation</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -334,8 +437,43 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="26">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -433,8 +571,56 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E75B6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBF8F00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEEAF6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBE4E4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -481,12 +667,97 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -538,20 +809,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -566,23 +825,92 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="24" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="25" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -898,146 +1226,146 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="30" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B3" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="37" t="s">
+      <c r="D3" s="34" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B3" s="22" t="s">
+      <c r="E3" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="F3" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="22" t="s">
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B4" s="34"/>
+      <c r="C4" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="35" t="s">
+      <c r="D4" s="34"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="36"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B5" s="34"/>
+      <c r="C5" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="38" t="s">
+      <c r="D5" s="34"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="36"/>
+    </row>
+    <row r="6" spans="2:6" ht="87" x14ac:dyDescent="0.35">
+      <c r="B6" s="34"/>
+      <c r="C6" s="23" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B4" s="22"/>
-      <c r="C4" s="25" t="s">
+      <c r="D6" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="38"/>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B5" s="22"/>
-      <c r="C5" s="26" t="s">
+      <c r="E6" s="35"/>
+      <c r="F6" s="36"/>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B7" s="34"/>
+      <c r="C7" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="38"/>
-    </row>
-    <row r="6" spans="2:6" ht="87" x14ac:dyDescent="0.35">
-      <c r="B6" s="22"/>
-      <c r="C6" s="27" t="s">
+      <c r="D7" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="E7" s="35"/>
+      <c r="F7" s="36"/>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B8" s="34"/>
+      <c r="C8" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="35"/>
-      <c r="F6" s="38"/>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B7" s="22"/>
-      <c r="C7" s="26" t="s">
+      <c r="D8" s="34"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="36"/>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B9" s="34"/>
+      <c r="C9" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D9" s="34"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="36"/>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B10" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="35"/>
-      <c r="F7" s="38"/>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B8" s="22"/>
-      <c r="C8" s="28" t="s">
+      <c r="C10" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="22"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="38"/>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B9" s="22"/>
-      <c r="C9" s="29" t="s">
+      <c r="D10" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="22"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="38"/>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B10" s="22" t="s">
+      <c r="E10" s="35"/>
+      <c r="F10" s="36"/>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B11" s="34"/>
+      <c r="C11" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="D11" s="34"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="36"/>
+    </row>
+    <row r="12" spans="2:6" ht="58" x14ac:dyDescent="0.35">
+      <c r="B12" s="34"/>
+      <c r="C12" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D12" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="35"/>
-      <c r="F10" s="38"/>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B11" s="22"/>
-      <c r="C11" s="31" t="s">
+      <c r="E12" s="35"/>
+      <c r="F12" s="36"/>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B13" s="34"/>
+      <c r="C13" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="38"/>
-    </row>
-    <row r="12" spans="2:6" ht="58" x14ac:dyDescent="0.35">
-      <c r="B12" s="22"/>
-      <c r="C12" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="E12" s="35"/>
-      <c r="F12" s="38"/>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B13" s="22"/>
-      <c r="C13" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="D13" s="22"/>
+      <c r="D13" s="34"/>
       <c r="E13" s="35"/>
-      <c r="F13" s="38"/>
+      <c r="F13" s="36"/>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="E14" s="36"/>
+      <c r="E14" s="29"/>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="33" t="s">
-        <v>54</v>
-      </c>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
+        <v>50</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1070,13 +1398,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
     </row>
     <row r="2" spans="1:5" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="1"/>
@@ -1282,24 +1610,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
     </row>
     <row r="2" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="21"/>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
+      <c r="A2" s="39"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
     </row>
     <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
@@ -1443,7 +1771,7 @@
         <v>21</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.35">
@@ -1456,8 +1784,8 @@
       <c r="D4" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="22" t="s">
-        <v>29</v>
+      <c r="E4" s="34" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.35">
@@ -1470,7 +1798,7 @@
       <c r="D5" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="22"/>
+      <c r="E5" s="34"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="14">
@@ -1482,8 +1810,8 @@
       <c r="D6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="17" t="s">
-        <v>30</v>
+      <c r="E6" s="19" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1492,4 +1820,152 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C75D32B-3DD8-45CD-93CC-94611D54B3F4}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="19.453125" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" customWidth="1"/>
+    <col min="4" max="4" width="21.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="41" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="42" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="43" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="180" x14ac:dyDescent="0.35">
+      <c r="A2" s="54" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="44" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="90" x14ac:dyDescent="0.35">
+      <c r="A3" s="53"/>
+      <c r="B3" s="45" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="44" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" s="45" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="32" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="55"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="47" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="46"/>
+    </row>
+    <row r="5" spans="1:4" ht="280" x14ac:dyDescent="0.35">
+      <c r="A5" s="54" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="56" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="44" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="95" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="55"/>
+      <c r="B6" s="57"/>
+      <c r="C6" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="47" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="340.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7" s="49" t="s">
+        <v>74</v>
+      </c>
+      <c r="C7" s="49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" s="49" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="290.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="48" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="49" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" s="49" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="49" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="250.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="48" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="49" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" s="49" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" s="49" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="40.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="48" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="50" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" s="51" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10" s="52" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update data from April 2026 Excel file
https://claude.ai/code/session_012KajSB15QHs2faZ4YuFhrV
</commit_message>
<xml_diff>
--- a/iirs_app/uploads/latest.xlsx
+++ b/iirs_app/uploads/latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Rino\LEARNING\SESMU_15_2026\FINAL_PROJECT\TUGAS\130526\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3808BA66-E405-4F99-A000-D2310CF6DE10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{850F6428-7DC5-4DCA-A39A-C9D732882AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="4" xr2:uid="{D9861903-4DD6-443F-BDCB-8CE2F4A777AE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="2" xr2:uid="{D9861903-4DD6-443F-BDCB-8CE2F4A777AE}"/>
   </bookViews>
   <sheets>
     <sheet name="GET THINGS DONE!" sheetId="4" r:id="rId1"/>
@@ -831,6 +831,45 @@
     <xf numFmtId="0" fontId="8" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="24" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="25" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -858,49 +897,10 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="19" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="22" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="24" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="25" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="22" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="22" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1226,132 +1226,132 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
       <c r="F2" s="30" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="47" t="s">
         <v>30</v>
       </c>
       <c r="C3" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="35" t="s">
+      <c r="E3" s="48" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="36" t="s">
+      <c r="F3" s="49" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B4" s="34"/>
+      <c r="B4" s="47"/>
       <c r="C4" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="34"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="36"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="49"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B5" s="34"/>
+      <c r="B5" s="47"/>
       <c r="C5" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="34"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="36"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="49"/>
     </row>
     <row r="6" spans="2:6" ht="87" x14ac:dyDescent="0.35">
-      <c r="B6" s="34"/>
+      <c r="B6" s="47"/>
       <c r="C6" s="23" t="s">
         <v>37</v>
       </c>
       <c r="D6" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="35"/>
-      <c r="F6" s="36"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="49"/>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B7" s="34"/>
+      <c r="B7" s="47"/>
       <c r="C7" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="D7" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="35"/>
-      <c r="F7" s="36"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="49"/>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B8" s="34"/>
+      <c r="B8" s="47"/>
       <c r="C8" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="34"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="36"/>
+      <c r="D8" s="47"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="49"/>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B9" s="34"/>
+      <c r="B9" s="47"/>
       <c r="C9" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="34"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="36"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="49"/>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="47" t="s">
         <v>43</v>
       </c>
       <c r="C10" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="34" t="s">
+      <c r="D10" s="47" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="35"/>
-      <c r="F10" s="36"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="49"/>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B11" s="34"/>
+      <c r="B11" s="47"/>
       <c r="C11" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="34"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="36"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="49"/>
     </row>
     <row r="12" spans="2:6" ht="58" x14ac:dyDescent="0.35">
-      <c r="B12" s="34"/>
+      <c r="B12" s="47"/>
       <c r="C12" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="34" t="s">
+      <c r="D12" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="35"/>
-      <c r="F12" s="36"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="49"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B13" s="34"/>
+      <c r="B13" s="47"/>
       <c r="C13" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="D13" s="34"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="36"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="49"/>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.35">
       <c r="E14" s="29"/>
@@ -1360,12 +1360,12 @@
       <c r="B15" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="31" t="s">
+      <c r="C15" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="32"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1398,13 +1398,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
     </row>
     <row r="2" spans="1:5" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="1"/>
@@ -1610,24 +1610,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
     </row>
     <row r="2" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="39"/>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
+      <c r="A2" s="52"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
     </row>
     <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
@@ -1688,8 +1688,8 @@
         <v>46.7</v>
       </c>
       <c r="D5" s="5">
-        <f t="shared" ref="D5:D6" si="1">(0.35*B5)+(0.65*C5)</f>
-        <v>34.940000000000005</v>
+        <f>(0.4*B5)+(0.6*C5)</f>
+        <v>33.26</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1" t="str">
@@ -1711,8 +1711,8 @@
         <v>45.1</v>
       </c>
       <c r="D6" s="5">
-        <f t="shared" si="1"/>
-        <v>38.3765</v>
+        <f>(0.4*B6)+(0.6*C6)</f>
+        <v>37.415999999999997</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1" t="str">
@@ -1784,7 +1784,7 @@
       <c r="D4" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="34" t="s">
+      <c r="E4" s="47" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       <c r="D5" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="34"/>
+      <c r="E5" s="47"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="14">
@@ -1832,131 +1832,131 @@
     <col min="4" max="4" width="21.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:4" ht="21.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="31" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="34" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="180" x14ac:dyDescent="0.35">
-      <c r="A2" s="54" t="s">
+    <row r="2" spans="1:4" ht="70" x14ac:dyDescent="0.35">
+      <c r="A2" s="53" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="D2" s="44" t="s">
+      <c r="D2" s="35" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="90" x14ac:dyDescent="0.35">
-      <c r="A3" s="53"/>
-      <c r="B3" s="45" t="s">
+    <row r="3" spans="1:4" ht="50" x14ac:dyDescent="0.35">
+      <c r="A3" s="54"/>
+      <c r="B3" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="36" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="32" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" ht="21.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="55"/>
-      <c r="B4" s="46"/>
-      <c r="C4" s="47" t="s">
+      <c r="B4" s="37"/>
+      <c r="C4" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="46"/>
-    </row>
-    <row r="5" spans="1:4" ht="280" x14ac:dyDescent="0.35">
-      <c r="A5" s="54" t="s">
+      <c r="D4" s="37"/>
+    </row>
+    <row r="5" spans="1:4" ht="100" x14ac:dyDescent="0.35">
+      <c r="A5" s="53" t="s">
         <v>67</v>
       </c>
       <c r="B5" s="56" t="s">
         <v>68</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="35" t="s">
         <v>69</v>
       </c>
-      <c r="D5" s="44" t="s">
+      <c r="D5" s="35" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="95" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="55"/>
       <c r="B6" s="57"/>
-      <c r="C6" s="47" t="s">
+      <c r="C6" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="47" t="s">
+      <c r="D6" s="38" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="340.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="48" t="s">
+    <row r="7" spans="1:4" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="49" t="s">
+      <c r="B7" s="40" t="s">
         <v>74</v>
       </c>
-      <c r="C7" s="49" t="s">
+      <c r="C7" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="D7" s="49" t="s">
+      <c r="D7" s="40" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="290.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="48" t="s">
+    <row r="8" spans="1:4" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="39" t="s">
         <v>77</v>
       </c>
-      <c r="B8" s="49" t="s">
+      <c r="B8" s="40" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="49" t="s">
+      <c r="C8" s="40" t="s">
         <v>79</v>
       </c>
-      <c r="D8" s="49" t="s">
+      <c r="D8" s="40" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="250.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="48" t="s">
+    <row r="9" spans="1:4" ht="80.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="39" t="s">
         <v>81</v>
       </c>
-      <c r="B9" s="49" t="s">
+      <c r="B9" s="40" t="s">
         <v>82</v>
       </c>
-      <c r="C9" s="49" t="s">
+      <c r="C9" s="40" t="s">
         <v>83</v>
       </c>
-      <c r="D9" s="49" t="s">
+      <c r="D9" s="40" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="40.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="48" t="s">
+    <row r="10" spans="1:4" ht="20.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="39" t="s">
         <v>85</v>
       </c>
-      <c r="B10" s="50" t="s">
+      <c r="B10" s="41" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="51" t="s">
+      <c r="C10" s="42" t="s">
         <v>87</v>
       </c>
-      <c r="D10" s="52" t="s">
+      <c r="D10" s="43" t="s">
         <v>88</v>
       </c>
     </row>

</xml_diff>